<commit_message>
Actualización automática del inventario, Google Sheets y productos.json
</commit_message>
<xml_diff>
--- a/inventario.xlsx
+++ b/inventario.xlsx
@@ -744,7 +744,7 @@
         <v>200000</v>
       </c>
       <c r="F8" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="G8" t="n">
         <v>1</v>
@@ -758,7 +758,7 @@
         <v/>
       </c>
       <c r="J8" t="n">
-        <v>270000</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="9">

</xml_diff>